<commit_message>
chore: backup company tracking artifacts
</commit_message>
<xml_diff>
--- a/watchlists/a_share_company_watchlist.xlsx
+++ b/watchlists/a_share_company_watchlist.xlsx
@@ -594,7 +594,7 @@
         <v>46151</v>
       </c>
       <c r="M2" s="4" t="n">
-        <v>46151</v>
+        <v>46153</v>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
@@ -660,7 +660,7 @@
         <v>46151</v>
       </c>
       <c r="M3" s="4" t="n">
-        <v>46151</v>
+        <v>46153</v>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
@@ -726,7 +726,7 @@
         <v>46151</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>46151</v>
+        <v>46153</v>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
@@ -792,7 +792,7 @@
         <v>46151</v>
       </c>
       <c r="M5" s="4" t="n">
-        <v>46151</v>
+        <v>46153</v>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
@@ -858,7 +858,7 @@
         <v>46151</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>46151</v>
+        <v>46153</v>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
@@ -924,7 +924,7 @@
         <v>46151</v>
       </c>
       <c r="M7" s="4" t="n">
-        <v>46151</v>
+        <v>46153</v>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
@@ -990,7 +990,7 @@
         <v>46151</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>46151</v>
+        <v>46153</v>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
@@ -1056,7 +1056,7 @@
         <v>46151</v>
       </c>
       <c r="M9" s="4" t="n">
-        <v>46151</v>
+        <v>46153</v>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
@@ -1122,7 +1122,7 @@
         <v>46151</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>46151</v>
+        <v>46153</v>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
chore: backup company tracking updates
</commit_message>
<xml_diff>
--- a/watchlists/a_share_company_watchlist.xlsx
+++ b/watchlists/a_share_company_watchlist.xlsx
@@ -11,7 +11,7 @@
     <sheet name="schema" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'watchlist'!$A$1:$N$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'watchlist'!$A$1:$N$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'schema'!$A$1:$C$15</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N10"/>
+  <dimension ref="A1:N11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -594,7 +594,7 @@
         <v>46151</v>
       </c>
       <c r="M2" s="4" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
@@ -660,7 +660,7 @@
         <v>46151</v>
       </c>
       <c r="M3" s="4" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
@@ -726,7 +726,7 @@
         <v>46151</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
@@ -792,7 +792,7 @@
         <v>46151</v>
       </c>
       <c r="M5" s="4" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
@@ -858,7 +858,7 @@
         <v>46151</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
@@ -924,7 +924,7 @@
         <v>46151</v>
       </c>
       <c r="M7" s="4" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
@@ -990,7 +990,7 @@
         <v>46151</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
@@ -1056,7 +1056,7 @@
         <v>46151</v>
       </c>
       <c r="M9" s="4" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
@@ -1122,7 +1122,7 @@
         <v>46151</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
@@ -1130,8 +1130,70 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>688668.SH</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>SSE STAR</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>鼎通科技</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>鼎通科技; 东莞市鼎通精密科技股份有限公司; Dingtong Technology; Dingtong Precision; 688668; 高速通讯连接器; 铜缆连接; OSFP; QSFP-DD; 1.6T; 800G</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>高速连接器; 铜缆连接; AI服务器; 数据中心; 汽车连接器; 散热</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>鼎通科技 OR 688668 OR Dingtong Technology OR 高速连接器 OR 铜缆连接 OR OSFP OR 1.6T OR 800G</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>高速通讯连接器/铜缆连接、AI服务器与数据中心需求、1.6T/800G产品、客户验证、汽车连接器和散热业务、公告与订单进展</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>CNINFO; SSE STAR; 公司IR</t>
+        </is>
+      </c>
+      <c r="L11" s="4" t="n"/>
+      <c r="M11" s="4" t="n"/>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>added by user request; baseline pending</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N10"/>
+  <autoFilter ref="A1:N11"/>
   <dataValidations count="3">
     <dataValidation sqref="A2:A200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Y,N"</formula1>

</xml_diff>

<commit_message>
chore: update company tracking for 2026-05-15
</commit_message>
<xml_diff>
--- a/watchlists/a_share_company_watchlist.xlsx
+++ b/watchlists/a_share_company_watchlist.xlsx
@@ -593,8 +593,10 @@
       <c r="L2" s="4" t="n">
         <v>46151</v>
       </c>
-      <c r="M2" s="4" t="n">
-        <v>46156</v>
+      <c r="M2" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
@@ -659,8 +661,10 @@
       <c r="L3" s="4" t="n">
         <v>46151</v>
       </c>
-      <c r="M3" s="4" t="n">
-        <v>46156</v>
+      <c r="M3" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
@@ -725,8 +729,10 @@
       <c r="L4" s="4" t="n">
         <v>46151</v>
       </c>
-      <c r="M4" s="4" t="n">
-        <v>46156</v>
+      <c r="M4" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
@@ -791,8 +797,10 @@
       <c r="L5" s="4" t="n">
         <v>46151</v>
       </c>
-      <c r="M5" s="4" t="n">
-        <v>46156</v>
+      <c r="M5" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
@@ -857,8 +865,10 @@
       <c r="L6" s="4" t="n">
         <v>46151</v>
       </c>
-      <c r="M6" s="4" t="n">
-        <v>46156</v>
+      <c r="M6" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
@@ -923,8 +933,10 @@
       <c r="L7" s="4" t="n">
         <v>46151</v>
       </c>
-      <c r="M7" s="4" t="n">
-        <v>46156</v>
+      <c r="M7" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
@@ -989,8 +1001,10 @@
       <c r="L8" s="4" t="n">
         <v>46151</v>
       </c>
-      <c r="M8" s="4" t="n">
-        <v>46156</v>
+      <c r="M8" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
@@ -1055,8 +1069,10 @@
       <c r="L9" s="4" t="n">
         <v>46151</v>
       </c>
-      <c r="M9" s="4" t="n">
-        <v>46156</v>
+      <c r="M9" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
@@ -1121,8 +1137,10 @@
       <c r="L10" s="4" t="n">
         <v>46151</v>
       </c>
-      <c r="M10" s="4" t="n">
-        <v>46156</v>
+      <c r="M10" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
@@ -1187,8 +1205,10 @@
       <c r="L11" s="4" t="n">
         <v>46156</v>
       </c>
-      <c r="M11" s="4" t="n">
-        <v>46156</v>
+      <c r="M11" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
@@ -1253,8 +1273,10 @@
       <c r="L12" s="4" t="n">
         <v>46156</v>
       </c>
-      <c r="M12" s="4" t="n">
-        <v>46156</v>
+      <c r="M12" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
chore: backup company tracking 2026-05-16
</commit_message>
<xml_diff>
--- a/watchlists/a_share_company_watchlist.xlsx
+++ b/watchlists/a_share_company_watchlist.xlsx
@@ -595,7 +595,7 @@
       </c>
       <c r="M2" s="4" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -663,7 +663,7 @@
       </c>
       <c r="M3" s="4" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
@@ -731,7 +731,7 @@
       </c>
       <c r="M4" s="4" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="M6" s="4" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="M9" s="4" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="M10" s="4" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="M12" s="4" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore: backup tracking and earnings snapshots
</commit_message>
<xml_diff>
--- a/watchlists/a_share_company_watchlist.xlsx
+++ b/watchlists/a_share_company_watchlist.xlsx
@@ -595,7 +595,7 @@
       </c>
       <c r="M2" s="4" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -663,7 +663,7 @@
       </c>
       <c r="M3" s="4" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
@@ -731,7 +731,7 @@
       </c>
       <c r="M4" s="4" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="M6" s="4" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="M9" s="4" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="M10" s="4" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="M12" s="4" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">

</xml_diff>

<commit_message>
feat: add stock moat triad research skill
</commit_message>
<xml_diff>
--- a/watchlists/a_share_company_watchlist.xlsx
+++ b/watchlists/a_share_company_watchlist.xlsx
@@ -595,7 +595,7 @@
       </c>
       <c r="M2" s="4" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -663,7 +663,7 @@
       </c>
       <c r="M3" s="4" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
@@ -731,7 +731,7 @@
       </c>
       <c r="M4" s="4" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="M6" s="4" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="M9" s="4" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="M10" s="4" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="M12" s="4" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore: backup research tracking artifacts
</commit_message>
<xml_diff>
--- a/watchlists/a_share_company_watchlist.xlsx
+++ b/watchlists/a_share_company_watchlist.xlsx
@@ -593,10 +593,8 @@
       <c r="L2" s="4" t="n">
         <v>46151</v>
       </c>
-      <c r="M2" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-23</t>
-        </is>
+      <c r="M2" s="4" t="n">
+        <v>46166</v>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
@@ -661,10 +659,8 @@
       <c r="L3" s="4" t="n">
         <v>46151</v>
       </c>
-      <c r="M3" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-23</t>
-        </is>
+      <c r="M3" s="4" t="n">
+        <v>46166</v>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
@@ -729,10 +725,8 @@
       <c r="L4" s="4" t="n">
         <v>46151</v>
       </c>
-      <c r="M4" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-23</t>
-        </is>
+      <c r="M4" s="4" t="n">
+        <v>46166</v>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
@@ -797,10 +791,8 @@
       <c r="L5" s="4" t="n">
         <v>46151</v>
       </c>
-      <c r="M5" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-23</t>
-        </is>
+      <c r="M5" s="4" t="n">
+        <v>46166</v>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
@@ -865,10 +857,8 @@
       <c r="L6" s="4" t="n">
         <v>46151</v>
       </c>
-      <c r="M6" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-23</t>
-        </is>
+      <c r="M6" s="4" t="n">
+        <v>46166</v>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
@@ -933,10 +923,8 @@
       <c r="L7" s="4" t="n">
         <v>46151</v>
       </c>
-      <c r="M7" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-23</t>
-        </is>
+      <c r="M7" s="4" t="n">
+        <v>46166</v>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
@@ -1001,10 +989,8 @@
       <c r="L8" s="4" t="n">
         <v>46151</v>
       </c>
-      <c r="M8" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-23</t>
-        </is>
+      <c r="M8" s="4" t="n">
+        <v>46166</v>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
@@ -1069,10 +1055,8 @@
       <c r="L9" s="4" t="n">
         <v>46151</v>
       </c>
-      <c r="M9" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-23</t>
-        </is>
+      <c r="M9" s="4" t="n">
+        <v>46166</v>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
@@ -1137,10 +1121,8 @@
       <c r="L10" s="4" t="n">
         <v>46151</v>
       </c>
-      <c r="M10" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-23</t>
-        </is>
+      <c r="M10" s="4" t="n">
+        <v>46166</v>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
@@ -1205,10 +1187,8 @@
       <c r="L11" s="4" t="n">
         <v>46156</v>
       </c>
-      <c r="M11" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-23</t>
-        </is>
+      <c r="M11" s="4" t="n">
+        <v>46166</v>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
@@ -1273,10 +1253,8 @@
       <c r="L12" s="4" t="n">
         <v>46156</v>
       </c>
-      <c r="M12" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-23</t>
-        </is>
+      <c r="M12" s="4" t="n">
+        <v>46166</v>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
@@ -1343,10 +1321,8 @@
           <t>2026-05-23</t>
         </is>
       </c>
-      <c r="M13" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-23</t>
-        </is>
+      <c r="M13" s="4" t="n">
+        <v>46166</v>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
chore: backup tracking and earnings updates
</commit_message>
<xml_diff>
--- a/watchlists/a_share_company_watchlist.xlsx
+++ b/watchlists/a_share_company_watchlist.xlsx
@@ -593,8 +593,10 @@
       <c r="L2" s="4" t="n">
         <v>46151</v>
       </c>
-      <c r="M2" s="4" t="n">
-        <v>46166</v>
+      <c r="M2" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
@@ -659,8 +661,10 @@
       <c r="L3" s="4" t="n">
         <v>46151</v>
       </c>
-      <c r="M3" s="4" t="n">
-        <v>46166</v>
+      <c r="M3" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
@@ -725,8 +729,10 @@
       <c r="L4" s="4" t="n">
         <v>46151</v>
       </c>
-      <c r="M4" s="4" t="n">
-        <v>46166</v>
+      <c r="M4" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
@@ -791,8 +797,10 @@
       <c r="L5" s="4" t="n">
         <v>46151</v>
       </c>
-      <c r="M5" s="4" t="n">
-        <v>46166</v>
+      <c r="M5" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
@@ -857,8 +865,10 @@
       <c r="L6" s="4" t="n">
         <v>46151</v>
       </c>
-      <c r="M6" s="4" t="n">
-        <v>46166</v>
+      <c r="M6" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
@@ -923,8 +933,10 @@
       <c r="L7" s="4" t="n">
         <v>46151</v>
       </c>
-      <c r="M7" s="4" t="n">
-        <v>46166</v>
+      <c r="M7" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
@@ -989,8 +1001,10 @@
       <c r="L8" s="4" t="n">
         <v>46151</v>
       </c>
-      <c r="M8" s="4" t="n">
-        <v>46166</v>
+      <c r="M8" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
@@ -1055,8 +1069,10 @@
       <c r="L9" s="4" t="n">
         <v>46151</v>
       </c>
-      <c r="M9" s="4" t="n">
-        <v>46166</v>
+      <c r="M9" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
@@ -1121,8 +1137,10 @@
       <c r="L10" s="4" t="n">
         <v>46151</v>
       </c>
-      <c r="M10" s="4" t="n">
-        <v>46166</v>
+      <c r="M10" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
@@ -1187,8 +1205,10 @@
       <c r="L11" s="4" t="n">
         <v>46156</v>
       </c>
-      <c r="M11" s="4" t="n">
-        <v>46166</v>
+      <c r="M11" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
@@ -1253,8 +1273,10 @@
       <c r="L12" s="4" t="n">
         <v>46156</v>
       </c>
-      <c r="M12" s="4" t="n">
-        <v>46166</v>
+      <c r="M12" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
@@ -1321,8 +1343,10 @@
           <t>2026-05-23</t>
         </is>
       </c>
-      <c r="M13" s="4" t="n">
-        <v>46166</v>
+      <c r="M13" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
chore: full backup 2026-05-31
</commit_message>
<xml_diff>
--- a/watchlists/a_share_company_watchlist.xlsx
+++ b/watchlists/a_share_company_watchlist.xlsx
@@ -595,7 +595,7 @@
       </c>
       <c r="M2" s="4" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -663,7 +663,7 @@
       </c>
       <c r="M3" s="4" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
@@ -731,7 +731,7 @@
       </c>
       <c r="M4" s="4" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="M6" s="4" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="M9" s="4" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="M10" s="4" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="M12" s="4" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -1345,7 +1345,7 @@
       </c>
       <c r="M13" s="4" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore: update company tracking 2026-06-01
</commit_message>
<xml_diff>
--- a/watchlists/a_share_company_watchlist.xlsx
+++ b/watchlists/a_share_company_watchlist.xlsx
@@ -595,7 +595,7 @@
       </c>
       <c r="M2" s="4" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -663,7 +663,7 @@
       </c>
       <c r="M3" s="4" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
@@ -731,7 +731,7 @@
       </c>
       <c r="M4" s="4" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="M6" s="4" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="M9" s="4" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="M10" s="4" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="M12" s="4" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -1345,7 +1345,7 @@
       </c>
       <c r="M13" s="4" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore: update A-share company tracking run
</commit_message>
<xml_diff>
--- a/watchlists/a_share_company_watchlist.xlsx
+++ b/watchlists/a_share_company_watchlist.xlsx
@@ -595,7 +595,7 @@
       </c>
       <c r="M2" s="4" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -663,7 +663,7 @@
       </c>
       <c r="M3" s="4" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
@@ -731,7 +731,7 @@
       </c>
       <c r="M4" s="4" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="M6" s="4" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="M9" s="4" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="M10" s="4" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="M12" s="4" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -1345,7 +1345,7 @@
       </c>
       <c r="M13" s="4" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore: update tracking run and earnings snapshot
</commit_message>
<xml_diff>
--- a/watchlists/a_share_company_watchlist.xlsx
+++ b/watchlists/a_share_company_watchlist.xlsx
@@ -595,7 +595,7 @@
       </c>
       <c r="M2" s="4" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -663,7 +663,7 @@
       </c>
       <c r="M3" s="4" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
@@ -731,7 +731,7 @@
       </c>
       <c r="M4" s="4" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="M6" s="4" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="M9" s="4" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="M10" s="4" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="M12" s="4" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -1345,7 +1345,7 @@
       </c>
       <c r="M13" s="4" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore: update tracking artifacts and earnings snapshot
</commit_message>
<xml_diff>
--- a/watchlists/a_share_company_watchlist.xlsx
+++ b/watchlists/a_share_company_watchlist.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N13"/>
+  <dimension ref="A1:N14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -595,7 +595,7 @@
       </c>
       <c r="M2" s="4" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -607,7 +607,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -668,14 +668,14 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>baseline created by parallel company deep research run</t>
+          <t>baseline created by parallel company deep research run; paused by user request on 2026-06-08; keep historical baseline/events but exclude from daily tracking</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -736,7 +736,7 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>baseline created by parallel company deep research run</t>
+          <t>baseline created by parallel company deep research run; paused by user request on 2026-06-08; keep historical baseline/events but exclude from daily tracking</t>
         </is>
       </c>
     </row>
@@ -799,7 +799,7 @@
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="M6" s="4" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="M9" s="4" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="M10" s="4" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="M12" s="4" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -1287,7 +1287,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -1350,7 +1350,75 @@
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>baseline created by 2026-05-23 company tracking controller fallback after worker timeout</t>
+          <t>baseline created by 2026-05-23 company tracking controller fallback after worker timeout; paused by user request on 2026-06-08; keep historical baseline/events but exclude from daily tracking</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>002851.SZ</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>SZSE</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>麦格米特</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>麦格米特; Megmeet; Shenzhen Megmeet; 002851; 数据中心电源; 800VDC; Power Shelf; BBU; AI服务器电源</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>数据中心电源; AI服务器电源; 800VDC; Power Shelf; BBU; 电力电子</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>麦格米特 OR 002851 OR Megmeet OR 800VDC OR Power Shelf OR BBU OR 数据中心电源</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>AI数据中心电源、800VDC/Power Shelf/BBU进展、海外客户验证、收入占比、毛利率和费用释放、公告与订单进展</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>CNINFO; SZSE; 公司IR; 公司官网</t>
+        </is>
+      </c>
+      <c r="L14" s="4" t="n">
+        <v>46181</v>
+      </c>
+      <c r="M14" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>added by user request on 2026-06-08; build baseline on next company-tracking run</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update company tracking backup artifacts
</commit_message>
<xml_diff>
--- a/watchlists/a_share_company_watchlist.xlsx
+++ b/watchlists/a_share_company_watchlist.xlsx
@@ -595,7 +595,7 @@
       </c>
       <c r="M2" s="4" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="M6" s="4" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="M9" s="4" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="M10" s="4" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="M12" s="4" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -1413,7 +1413,7 @@
       </c>
       <c r="M14" s="4" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore: update company tracking run artifacts
</commit_message>
<xml_diff>
--- a/watchlists/a_share_company_watchlist.xlsx
+++ b/watchlists/a_share_company_watchlist.xlsx
@@ -595,7 +595,7 @@
       </c>
       <c r="M2" s="4" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="M6" s="4" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="M9" s="4" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="M10" s="4" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="M12" s="4" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -1413,7 +1413,7 @@
       </c>
       <c r="M14" s="4" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore: update A-share company tracking
</commit_message>
<xml_diff>
--- a/watchlists/a_share_company_watchlist.xlsx
+++ b/watchlists/a_share_company_watchlist.xlsx
@@ -595,7 +595,7 @@
       </c>
       <c r="M2" s="4" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="M6" s="4" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="M9" s="4" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="M10" s="4" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="M12" s="4" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -1413,7 +1413,7 @@
       </c>
       <c r="M14" s="4" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">

</xml_diff>

<commit_message>
docs: update industry chain research artifacts
</commit_message>
<xml_diff>
--- a/watchlists/a_share_company_watchlist.xlsx
+++ b/watchlists/a_share_company_watchlist.xlsx
@@ -595,7 +595,7 @@
       </c>
       <c r="M2" s="4" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="M6" s="4" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="M9" s="4" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="M10" s="4" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="M12" s="4" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -1413,7 +1413,7 @@
       </c>
       <c r="M14" s="4" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">

</xml_diff>

<commit_message>
docs: update a-share tracking artifacts
</commit_message>
<xml_diff>
--- a/watchlists/a_share_company_watchlist.xlsx
+++ b/watchlists/a_share_company_watchlist.xlsx
@@ -595,7 +595,7 @@
       </c>
       <c r="M2" s="4" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="M6" s="4" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="M9" s="4" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="M10" s="4" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="M12" s="4" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -1413,7 +1413,7 @@
       </c>
       <c r="M14" s="4" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">

</xml_diff>

<commit_message>
data: update A-share company tracking for 2026-06-18
</commit_message>
<xml_diff>
--- a/watchlists/a_share_company_watchlist.xlsx
+++ b/watchlists/a_share_company_watchlist.xlsx
@@ -595,7 +595,7 @@
       </c>
       <c r="M2" s="4" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="M6" s="4" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="M9" s="4" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="M10" s="4" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="M12" s="4" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -1413,7 +1413,7 @@
       </c>
       <c r="M14" s="4" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">

</xml_diff>

<commit_message>
docs: update A-share tracking for 2026-06-19
</commit_message>
<xml_diff>
--- a/watchlists/a_share_company_watchlist.xlsx
+++ b/watchlists/a_share_company_watchlist.xlsx
@@ -595,7 +595,7 @@
       </c>
       <c r="M2" s="4" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="M6" s="4" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="M9" s="4" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="M10" s="4" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="M12" s="4" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -1413,7 +1413,7 @@
       </c>
       <c r="M14" s="4" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">

</xml_diff>

<commit_message>
data: backup A-share tracking for 2026-06-22
</commit_message>
<xml_diff>
--- a/watchlists/a_share_company_watchlist.xlsx
+++ b/watchlists/a_share_company_watchlist.xlsx
@@ -595,7 +595,7 @@
       </c>
       <c r="M2" s="4" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="M6" s="4" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="M9" s="4" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="M10" s="4" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="M12" s="4" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -1413,7 +1413,7 @@
       </c>
       <c r="M14" s="4" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore: backup company tracking 2026-06-23
</commit_message>
<xml_diff>
--- a/watchlists/a_share_company_watchlist.xlsx
+++ b/watchlists/a_share_company_watchlist.xlsx
@@ -595,7 +595,7 @@
       </c>
       <c r="M2" s="4" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="M6" s="4" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="M9" s="4" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="M10" s="4" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="M12" s="4" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -1413,7 +1413,7 @@
       </c>
       <c r="M14" s="4" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore: full backup fund tracking and company updates
</commit_message>
<xml_diff>
--- a/watchlists/a_share_company_watchlist.xlsx
+++ b/watchlists/a_share_company_watchlist.xlsx
@@ -595,7 +595,7 @@
       </c>
       <c r="M2" s="4" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="M6" s="4" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="M9" s="4" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="M10" s="4" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="M12" s="4" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -1413,7 +1413,7 @@
       </c>
       <c r="M14" s="4" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore: full backup company and tungsten tracking
</commit_message>
<xml_diff>
--- a/watchlists/a_share_company_watchlist.xlsx
+++ b/watchlists/a_share_company_watchlist.xlsx
@@ -595,7 +595,7 @@
       </c>
       <c r="M2" s="4" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="M6" s="4" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="M9" s="4" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="M10" s="4" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="M12" s="4" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -1413,7 +1413,7 @@
       </c>
       <c r="M14" s="4" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore: full backup company tracking updates
</commit_message>
<xml_diff>
--- a/watchlists/a_share_company_watchlist.xlsx
+++ b/watchlists/a_share_company_watchlist.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="watchlist" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="schema" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="watchlist" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="schema" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'watchlist'!$A$1:$N$11</definedName>
@@ -595,7 +595,7 @@
       </c>
       <c r="M2" s="4" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="M6" s="4" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="M9" s="4" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="M10" s="4" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="M12" s="4" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -1413,7 +1413,7 @@
       </c>
       <c r="M14" s="4" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore: full backup tracking updates
</commit_message>
<xml_diff>
--- a/watchlists/a_share_company_watchlist.xlsx
+++ b/watchlists/a_share_company_watchlist.xlsx
@@ -595,7 +595,7 @@
       </c>
       <c r="M2" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="M6" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="M9" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="M10" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="M12" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -1413,7 +1413,7 @@
       </c>
       <c r="M14" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore: full backup 2026-07-02 tracking updates
</commit_message>
<xml_diff>
--- a/watchlists/a_share_company_watchlist.xlsx
+++ b/watchlists/a_share_company_watchlist.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N14"/>
+  <dimension ref="A1:N15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -595,7 +595,7 @@
       </c>
       <c r="M2" s="4" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="M6" s="4" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="M9" s="4" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="M10" s="4" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="M12" s="4" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -1413,12 +1413,78 @@
       </c>
       <c r="M14" s="4" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
           <t>added by user request on 2026-06-08; build baseline on next company-tracking run</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>000636.SZ</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>SZSE</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>风华高科</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>风华高科; 广东风华高新科技股份有限公司; Guangdong Fenghua Advanced Technology Holding Co.,Ltd.; FENGHUA; FHAT; 000636; MLCC; 高容MLCC; 片式电容; 片式电阻; 电感; 被动元件</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>MLCC; 高端被动元件; 电子元器件; 电子材料; AI算力; 车规; 工控</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>风华高科 OR 000636 OR MLCC OR 高容MLCC OR 片式电阻 OR 电感 OR AI算力 OR 英伟达认证</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>高容/高温/高可靠MLCC、AI算力被动元件、客户编码和批量交付、收入占比、ASP、毛利率、龙虎榜和大宗交易拥挤度</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>公司官网; CNINFO; SZSE; 公司IR; 交易所公开交易信息; 东方财富/AKShare交易数据交叉核对</t>
+        </is>
+      </c>
+      <c r="L15" s="4" t="n">
+        <v>46205</v>
+      </c>
+      <c r="M15" s="4" t="n">
+        <v>46205</v>
+      </c>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>added by user request on 2026-07-02; full baseline built on 2026-07-02; strict boundary: official disclosures deny direct NVIDIA supply/certification; track AI high-end MLCC evidence separately from trading heat</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: full backup 2026-07-03 tracking updates
</commit_message>
<xml_diff>
--- a/watchlists/a_share_company_watchlist.xlsx
+++ b/watchlists/a_share_company_watchlist.xlsx
@@ -595,7 +595,7 @@
       </c>
       <c r="M2" s="4" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="M6" s="4" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="M9" s="4" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="M10" s="4" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="M12" s="4" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -1413,7 +1413,7 @@
       </c>
       <c r="M14" s="4" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
@@ -1479,8 +1479,10 @@
       <c r="L15" s="4" t="n">
         <v>46205</v>
       </c>
-      <c r="M15" s="4" t="n">
-        <v>46205</v>
+      <c r="M15" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
chore: full backup 2026-07-06 company tracking
</commit_message>
<xml_diff>
--- a/watchlists/a_share_company_watchlist.xlsx
+++ b/watchlists/a_share_company_watchlist.xlsx
@@ -595,7 +595,7 @@
       </c>
       <c r="M2" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="M6" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="M9" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="M10" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="M12" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -1413,7 +1413,7 @@
       </c>
       <c r="M14" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
@@ -1481,7 +1481,7 @@
       </c>
       <c r="M15" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore: full backup 2026-07-07 tracking updates
</commit_message>
<xml_diff>
--- a/watchlists/a_share_company_watchlist.xlsx
+++ b/watchlists/a_share_company_watchlist.xlsx
@@ -595,7 +595,7 @@
       </c>
       <c r="M2" s="4" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="M6" s="4" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="M9" s="4" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="M10" s="4" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="M12" s="4" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -1413,7 +1413,7 @@
       </c>
       <c r="M14" s="4" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
@@ -1481,7 +1481,7 @@
       </c>
       <c r="M15" s="4" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore: full backup 2026-07-08 tracking updates
</commit_message>
<xml_diff>
--- a/watchlists/a_share_company_watchlist.xlsx
+++ b/watchlists/a_share_company_watchlist.xlsx
@@ -595,7 +595,7 @@
       </c>
       <c r="M2" s="4" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="M6" s="4" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="M9" s="4" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="M10" s="4" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="M12" s="4" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -1413,7 +1413,7 @@
       </c>
       <c r="M14" s="4" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
@@ -1481,7 +1481,7 @@
       </c>
       <c r="M15" s="4" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore: backup company tracking 2026-07-09
</commit_message>
<xml_diff>
--- a/watchlists/a_share_company_watchlist.xlsx
+++ b/watchlists/a_share_company_watchlist.xlsx
@@ -595,7 +595,7 @@
       </c>
       <c r="M2" s="4" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="M6" s="4" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="M9" s="4" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="M10" s="4" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="M12" s="4" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -1413,7 +1413,7 @@
       </c>
       <c r="M14" s="4" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
@@ -1481,7 +1481,7 @@
       </c>
       <c r="M15" s="4" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore: full backup 2026-07-10 company tracking
</commit_message>
<xml_diff>
--- a/watchlists/a_share_company_watchlist.xlsx
+++ b/watchlists/a_share_company_watchlist.xlsx
@@ -595,7 +595,7 @@
       </c>
       <c r="M2" s="4" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="M6" s="4" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="M9" s="4" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="M10" s="4" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="M12" s="4" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -1413,7 +1413,7 @@
       </c>
       <c r="M14" s="4" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
@@ -1481,7 +1481,7 @@
       </c>
       <c r="M15" s="4" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore: full backup 2026-07-14 research updates
</commit_message>
<xml_diff>
--- a/watchlists/a_share_company_watchlist.xlsx
+++ b/watchlists/a_share_company_watchlist.xlsx
@@ -595,7 +595,7 @@
       </c>
       <c r="M2" s="4" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="M6" s="4" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="M9" s="4" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="M10" s="4" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="M12" s="4" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -1413,7 +1413,7 @@
       </c>
       <c r="M14" s="4" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
@@ -1481,7 +1481,7 @@
       </c>
       <c r="M15" s="4" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore: backup company tracking 2026-07-16
</commit_message>
<xml_diff>
--- a/watchlists/a_share_company_watchlist.xlsx
+++ b/watchlists/a_share_company_watchlist.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N15"/>
+  <dimension ref="A1:N17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -595,7 +595,7 @@
       </c>
       <c r="M2" s="4" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="M6" s="4" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="M9" s="4" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="M10" s="4" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="M12" s="4" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -1413,7 +1413,7 @@
       </c>
       <c r="M14" s="4" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
@@ -1481,12 +1481,144 @@
       </c>
       <c r="M15" s="4" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
           <t>added by user request on 2026-07-02; full baseline built on 2026-07-02; strict boundary: official disclosures deny direct NVIDIA supply/certification; track AI high-end MLCC evidence separately from trading heat</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>688048.SH</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>SSE STAR</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>长光华芯</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>长光华芯; 苏州长光华芯光电技术股份有限公司; Everbright Photonics; 688048; 半导体激光芯片; 高功率激光芯片; VCSEL; EML; DFB; 光通信芯片</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>半导体激光芯片; 高功率激光; VCSEL; EML; DFB; 光通信; 激光雷达</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>长光华芯 OR 688048 OR Everbright Photonics OR 高功率激光芯片 OR VCSEL OR EML OR DFB OR 光通信芯片</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>高功率半导体激光芯片、VCSEL/EML/DFB/PIN PD光通信产品、客户验证、批量出货、产能良率、扣非盈利和现金流</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>CNINFO; SSE STAR; 公司IR; 公司官网</t>
+        </is>
+      </c>
+      <c r="L16" s="4" t="n">
+        <v>46219</v>
+      </c>
+      <c r="M16" s="4" t="n">
+        <v>46219</v>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>added by user request on 2026-07-16; full baseline built on 2026-07-16; keep optical-communication market expansion and customer validation separate from confirmed orders/revenue</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>301217.SZ</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>SZSE</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>铜冠铜箔</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>铜冠铜箔; 安徽铜冠铜箔集团股份有限公司; Tongguan Copper Foil; TGCF; 301217; PCB铜箔; 锂电铜箔; HVLP; RTF</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>PCB铜箔; 锂电铜箔; 高频高速铜箔; HVLP; RTF; AI PCB材料</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>铜冠铜箔 OR 301217 OR Tongguan Copper Foil OR TGCF OR PCB铜箔 OR HVLP OR RTF OR AI PCB铜箔</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>PCB铜箔与锂电铜箔分产品产销、HVLP/RTF分代客户认证与批量交付、加工费、产能利用率、盈利和现金流</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>CNINFO; SZSE; 公司IR; 公司官网</t>
+        </is>
+      </c>
+      <c r="L17" s="4" t="n">
+        <v>46219</v>
+      </c>
+      <c r="M17" s="4" t="n">
+        <v>46219</v>
+      </c>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>added by user request on 2026-07-16; full baseline built on 2026-07-16; keep lithium-battery copper foil separate from AI PCB/high-frequency PCB copper foil</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: backup company tracking 2026-07-29
🤖 Generated with [Claude Code](https://claude.com/claude-code)

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/watchlists/a_share_company_watchlist.xlsx
+++ b/watchlists/a_share_company_watchlist.xlsx
@@ -595,7 +595,7 @@
       </c>
       <c r="M2" s="4" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="M6" s="4" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="M9" s="4" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="M10" s="4" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="M12" s="4" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -1413,7 +1413,7 @@
       </c>
       <c r="M14" s="4" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
@@ -1481,7 +1481,7 @@
       </c>
       <c r="M15" s="4" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
@@ -1548,7 +1548,7 @@
         <v>46219</v>
       </c>
       <c r="M16" s="4" t="n">
-        <v>46223</v>
+        <v>46232</v>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
@@ -1614,7 +1614,7 @@
         <v>46219</v>
       </c>
       <c r="M17" s="4" t="n">
-        <v>46223</v>
+        <v>46232</v>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
chore: full backup Kronos PIT remediation
</commit_message>
<xml_diff>
--- a/watchlists/a_share_company_watchlist.xlsx
+++ b/watchlists/a_share_company_watchlist.xlsx
@@ -595,7 +595,7 @@
       </c>
       <c r="M2" s="4" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="M6" s="4" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="M9" s="4" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="M10" s="4" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="M12" s="4" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -1413,7 +1413,7 @@
       </c>
       <c r="M14" s="4" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
@@ -1481,7 +1481,7 @@
       </c>
       <c r="M15" s="4" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
@@ -1549,7 +1549,7 @@
       </c>
       <c r="M16" s="4" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
@@ -1617,7 +1617,7 @@
       </c>
       <c r="M17" s="4" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore: remove Kronos skill and sync research tracking
</commit_message>
<xml_diff>
--- a/watchlists/a_share_company_watchlist.xlsx
+++ b/watchlists/a_share_company_watchlist.xlsx
@@ -595,7 +595,7 @@
       </c>
       <c r="M2" s="4" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="M6" s="4" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="M9" s="4" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="M10" s="4" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="M12" s="4" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -1413,7 +1413,7 @@
       </c>
       <c r="M14" s="4" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
@@ -1481,7 +1481,7 @@
       </c>
       <c r="M15" s="4" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
@@ -1549,7 +1549,7 @@
       </c>
       <c r="M16" s="4" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
@@ -1617,7 +1617,7 @@
       </c>
       <c r="M17" s="4" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Update A-share company tracking with 2026-08-10 trading data
</commit_message>
<xml_diff>
--- a/watchlists/a_share_company_watchlist.xlsx
+++ b/watchlists/a_share_company_watchlist.xlsx
@@ -595,7 +595,7 @@
       </c>
       <c r="M2" s="4" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="M6" s="4" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="M9" s="4" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="M10" s="4" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="M12" s="4" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -1413,7 +1413,7 @@
       </c>
       <c r="M14" s="4" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
@@ -1481,7 +1481,7 @@
       </c>
       <c r="M15" s="4" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
@@ -1549,7 +1549,7 @@
       </c>
       <c r="M16" s="4" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
@@ -1617,7 +1617,7 @@
       </c>
       <c r="M17" s="4" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Refresh tracking status and margin audit data
</commit_message>
<xml_diff>
--- a/watchlists/a_share_company_watchlist.xlsx
+++ b/watchlists/a_share_company_watchlist.xlsx
@@ -595,7 +595,7 @@
       </c>
       <c r="M2" s="4" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="M6" s="4" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="M9" s="4" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="M10" s="4" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="M12" s="4" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -1413,7 +1413,7 @@
       </c>
       <c r="M14" s="4" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
@@ -1481,7 +1481,7 @@
       </c>
       <c r="M15" s="4" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
@@ -1549,7 +1549,7 @@
       </c>
       <c r="M16" s="4" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
@@ -1617,7 +1617,7 @@
       </c>
       <c r="M17" s="4" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore: full backup 2026-08-12
🤖 Generated with [Claude Code](https://claude.com/claude-code)

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/watchlists/a_share_company_watchlist.xlsx
+++ b/watchlists/a_share_company_watchlist.xlsx
@@ -595,7 +595,7 @@
       </c>
       <c r="M2" s="4" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="M6" s="4" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="M9" s="4" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="M10" s="4" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="M12" s="4" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -1413,7 +1413,7 @@
       </c>
       <c r="M14" s="4" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
@@ -1481,7 +1481,7 @@
       </c>
       <c r="M15" s="4" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
@@ -1549,7 +1549,7 @@
       </c>
       <c r="M16" s="4" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
@@ -1617,7 +1617,7 @@
       </c>
       <c r="M17" s="4" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore: back up company tracking run 2026-08-13
</commit_message>
<xml_diff>
--- a/watchlists/a_share_company_watchlist.xlsx
+++ b/watchlists/a_share_company_watchlist.xlsx
@@ -595,7 +595,7 @@
       </c>
       <c r="M2" s="4" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="M6" s="4" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="M9" s="4" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="M10" s="4" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="M12" s="4" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -1413,7 +1413,7 @@
       </c>
       <c r="M14" s="4" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
@@ -1481,7 +1481,7 @@
       </c>
       <c r="M15" s="4" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
@@ -1549,7 +1549,7 @@
       </c>
       <c r="M16" s="4" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
@@ -1617,7 +1617,7 @@
       </c>
       <c r="M17" s="4" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore: back up company tracking run 2026-08-14
</commit_message>
<xml_diff>
--- a/watchlists/a_share_company_watchlist.xlsx
+++ b/watchlists/a_share_company_watchlist.xlsx
@@ -595,7 +595,7 @@
       </c>
       <c r="M2" s="4" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="M6" s="4" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="M9" s="4" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="M10" s="4" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="M12" s="4" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -1413,7 +1413,7 @@
       </c>
       <c r="M14" s="4" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
@@ -1481,7 +1481,7 @@
       </c>
       <c r="M15" s="4" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
@@ -1549,7 +1549,7 @@
       </c>
       <c r="M16" s="4" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
@@ -1617,7 +1617,7 @@
       </c>
       <c r="M17" s="4" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore: backup company tracking and earnings snapshots
</commit_message>
<xml_diff>
--- a/watchlists/a_share_company_watchlist.xlsx
+++ b/watchlists/a_share_company_watchlist.xlsx
@@ -593,10 +593,8 @@
       <c r="L2" s="4" t="n">
         <v>46151</v>
       </c>
-      <c r="M2" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-14</t>
-        </is>
+      <c r="M2" s="4" t="n">
+        <v>46254</v>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
@@ -797,10 +795,8 @@
       <c r="L5" s="4" t="n">
         <v>46151</v>
       </c>
-      <c r="M5" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-14</t>
-        </is>
+      <c r="M5" s="4" t="n">
+        <v>46254</v>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
@@ -865,10 +861,8 @@
       <c r="L6" s="4" t="n">
         <v>46151</v>
       </c>
-      <c r="M6" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-14</t>
-        </is>
+      <c r="M6" s="4" t="n">
+        <v>46254</v>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
@@ -933,10 +927,8 @@
       <c r="L7" s="4" t="n">
         <v>46151</v>
       </c>
-      <c r="M7" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-14</t>
-        </is>
+      <c r="M7" s="4" t="n">
+        <v>46254</v>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
@@ -1001,10 +993,8 @@
       <c r="L8" s="4" t="n">
         <v>46151</v>
       </c>
-      <c r="M8" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-14</t>
-        </is>
+      <c r="M8" s="4" t="n">
+        <v>46254</v>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
@@ -1069,10 +1059,8 @@
       <c r="L9" s="4" t="n">
         <v>46151</v>
       </c>
-      <c r="M9" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-14</t>
-        </is>
+      <c r="M9" s="4" t="n">
+        <v>46254</v>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
@@ -1137,10 +1125,8 @@
       <c r="L10" s="4" t="n">
         <v>46151</v>
       </c>
-      <c r="M10" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-14</t>
-        </is>
+      <c r="M10" s="4" t="n">
+        <v>46254</v>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
@@ -1205,10 +1191,8 @@
       <c r="L11" s="4" t="n">
         <v>46156</v>
       </c>
-      <c r="M11" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-14</t>
-        </is>
+      <c r="M11" s="4" t="n">
+        <v>46254</v>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
@@ -1273,10 +1257,8 @@
       <c r="L12" s="4" t="n">
         <v>46156</v>
       </c>
-      <c r="M12" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-14</t>
-        </is>
+      <c r="M12" s="4" t="n">
+        <v>46254</v>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
@@ -1411,10 +1393,8 @@
       <c r="L14" s="4" t="n">
         <v>46181</v>
       </c>
-      <c r="M14" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-14</t>
-        </is>
+      <c r="M14" s="4" t="n">
+        <v>46254</v>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
@@ -1479,10 +1459,8 @@
       <c r="L15" s="4" t="n">
         <v>46205</v>
       </c>
-      <c r="M15" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-14</t>
-        </is>
+      <c r="M15" s="4" t="n">
+        <v>46254</v>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
@@ -1547,10 +1525,8 @@
       <c r="L16" s="4" t="n">
         <v>46219</v>
       </c>
-      <c r="M16" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-14</t>
-        </is>
+      <c r="M16" s="4" t="n">
+        <v>46254</v>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
@@ -1615,10 +1591,8 @@
       <c r="L17" s="4" t="n">
         <v>46219</v>
       </c>
-      <c r="M17" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-14</t>
-        </is>
+      <c r="M17" s="4" t="n">
+        <v>46254</v>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
chore: full backup company tracking 2026-08-21
</commit_message>
<xml_diff>
--- a/watchlists/a_share_company_watchlist.xlsx
+++ b/watchlists/a_share_company_watchlist.xlsx
@@ -594,7 +594,7 @@
         <v>46151</v>
       </c>
       <c r="M2" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
@@ -796,7 +796,7 @@
         <v>46151</v>
       </c>
       <c r="M5" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
@@ -862,7 +862,7 @@
         <v>46151</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
@@ -928,7 +928,7 @@
         <v>46151</v>
       </c>
       <c r="M7" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
@@ -994,7 +994,7 @@
         <v>46151</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
@@ -1060,7 +1060,7 @@
         <v>46151</v>
       </c>
       <c r="M9" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
@@ -1126,7 +1126,7 @@
         <v>46151</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
@@ -1192,7 +1192,7 @@
         <v>46156</v>
       </c>
       <c r="M11" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
@@ -1258,7 +1258,7 @@
         <v>46156</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
@@ -1394,7 +1394,7 @@
         <v>46181</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
@@ -1460,7 +1460,7 @@
         <v>46205</v>
       </c>
       <c r="M15" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
@@ -1526,7 +1526,7 @@
         <v>46219</v>
       </c>
       <c r="M16" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
@@ -1592,7 +1592,7 @@
         <v>46219</v>
       </c>
       <c r="M17" s="4" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
chore: backup company tracking and earnings updates
</commit_message>
<xml_diff>
--- a/watchlists/a_share_company_watchlist.xlsx
+++ b/watchlists/a_share_company_watchlist.xlsx
@@ -594,7 +594,7 @@
         <v>46151</v>
       </c>
       <c r="M2" s="4" t="n">
-        <v>46255</v>
+        <v>46258</v>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
@@ -796,7 +796,7 @@
         <v>46151</v>
       </c>
       <c r="M5" s="4" t="n">
-        <v>46255</v>
+        <v>46258</v>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
@@ -862,7 +862,7 @@
         <v>46151</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>46255</v>
+        <v>46258</v>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
@@ -928,7 +928,7 @@
         <v>46151</v>
       </c>
       <c r="M7" s="4" t="n">
-        <v>46255</v>
+        <v>46258</v>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
@@ -994,7 +994,7 @@
         <v>46151</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>46255</v>
+        <v>46258</v>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
@@ -1060,7 +1060,7 @@
         <v>46151</v>
       </c>
       <c r="M9" s="4" t="n">
-        <v>46255</v>
+        <v>46258</v>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
@@ -1126,7 +1126,7 @@
         <v>46151</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>46255</v>
+        <v>46258</v>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
@@ -1192,7 +1192,7 @@
         <v>46156</v>
       </c>
       <c r="M11" s="4" t="n">
-        <v>46255</v>
+        <v>46258</v>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
@@ -1258,7 +1258,7 @@
         <v>46156</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>46255</v>
+        <v>46258</v>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
@@ -1394,7 +1394,7 @@
         <v>46181</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>46255</v>
+        <v>46258</v>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
@@ -1460,7 +1460,7 @@
         <v>46205</v>
       </c>
       <c r="M15" s="4" t="n">
-        <v>46255</v>
+        <v>46258</v>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
@@ -1526,7 +1526,7 @@
         <v>46219</v>
       </c>
       <c r="M16" s="4" t="n">
-        <v>46255</v>
+        <v>46258</v>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
@@ -1592,7 +1592,7 @@
         <v>46219</v>
       </c>
       <c r="M17" s="4" t="n">
-        <v>46255</v>
+        <v>46258</v>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
chore: full backup tracking and earnings runs 2026-08-25
</commit_message>
<xml_diff>
--- a/watchlists/a_share_company_watchlist.xlsx
+++ b/watchlists/a_share_company_watchlist.xlsx
@@ -594,7 +594,7 @@
         <v>46151</v>
       </c>
       <c r="M2" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
@@ -796,7 +796,7 @@
         <v>46151</v>
       </c>
       <c r="M5" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
@@ -862,7 +862,7 @@
         <v>46151</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
@@ -928,7 +928,7 @@
         <v>46151</v>
       </c>
       <c r="M7" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
@@ -994,7 +994,7 @@
         <v>46151</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
@@ -1060,7 +1060,7 @@
         <v>46151</v>
       </c>
       <c r="M9" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
@@ -1126,7 +1126,7 @@
         <v>46151</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
@@ -1192,7 +1192,7 @@
         <v>46156</v>
       </c>
       <c r="M11" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
@@ -1258,7 +1258,7 @@
         <v>46156</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
@@ -1394,7 +1394,7 @@
         <v>46181</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
@@ -1460,7 +1460,7 @@
         <v>46205</v>
       </c>
       <c r="M15" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
@@ -1526,7 +1526,7 @@
         <v>46219</v>
       </c>
       <c r="M16" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
@@ -1592,7 +1592,7 @@
         <v>46219</v>
       </c>
       <c r="M17" s="4" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
chore: back up full worktree 2026-08-27
</commit_message>
<xml_diff>
--- a/watchlists/a_share_company_watchlist.xlsx
+++ b/watchlists/a_share_company_watchlist.xlsx
@@ -594,7 +594,7 @@
         <v>46151</v>
       </c>
       <c r="M2" s="4" t="n">
-        <v>46259</v>
+        <v>46261</v>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
@@ -796,7 +796,7 @@
         <v>46151</v>
       </c>
       <c r="M5" s="4" t="n">
-        <v>46259</v>
+        <v>46261</v>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
@@ -862,7 +862,7 @@
         <v>46151</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>46259</v>
+        <v>46261</v>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
@@ -928,7 +928,7 @@
         <v>46151</v>
       </c>
       <c r="M7" s="4" t="n">
-        <v>46259</v>
+        <v>46261</v>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
@@ -994,7 +994,7 @@
         <v>46151</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>46259</v>
+        <v>46261</v>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
@@ -1060,7 +1060,7 @@
         <v>46151</v>
       </c>
       <c r="M9" s="4" t="n">
-        <v>46259</v>
+        <v>46261</v>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
@@ -1126,7 +1126,7 @@
         <v>46151</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>46259</v>
+        <v>46261</v>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
@@ -1192,7 +1192,7 @@
         <v>46156</v>
       </c>
       <c r="M11" s="4" t="n">
-        <v>46259</v>
+        <v>46261</v>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
@@ -1258,7 +1258,7 @@
         <v>46156</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>46259</v>
+        <v>46261</v>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
@@ -1394,7 +1394,7 @@
         <v>46181</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>46259</v>
+        <v>46261</v>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
@@ -1460,7 +1460,7 @@
         <v>46205</v>
       </c>
       <c r="M15" s="4" t="n">
-        <v>46259</v>
+        <v>46261</v>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
@@ -1526,7 +1526,7 @@
         <v>46219</v>
       </c>
       <c r="M16" s="4" t="n">
-        <v>46259</v>
+        <v>46261</v>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
@@ -1592,7 +1592,7 @@
         <v>46219</v>
       </c>
       <c r="M17" s="4" t="n">
-        <v>46259</v>
+        <v>46261</v>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
chore: backup company tracking 2026-08-28
</commit_message>
<xml_diff>
--- a/watchlists/a_share_company_watchlist.xlsx
+++ b/watchlists/a_share_company_watchlist.xlsx
@@ -594,7 +594,7 @@
         <v>46151</v>
       </c>
       <c r="M2" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
@@ -796,7 +796,7 @@
         <v>46151</v>
       </c>
       <c r="M5" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
@@ -862,7 +862,7 @@
         <v>46151</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
@@ -928,7 +928,7 @@
         <v>46151</v>
       </c>
       <c r="M7" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
@@ -994,7 +994,7 @@
         <v>46151</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
@@ -1060,7 +1060,7 @@
         <v>46151</v>
       </c>
       <c r="M9" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
@@ -1126,7 +1126,7 @@
         <v>46151</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
@@ -1192,7 +1192,7 @@
         <v>46156</v>
       </c>
       <c r="M11" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
@@ -1258,7 +1258,7 @@
         <v>46156</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
@@ -1394,7 +1394,7 @@
         <v>46181</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
@@ -1460,7 +1460,7 @@
         <v>46205</v>
       </c>
       <c r="M15" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
@@ -1526,7 +1526,7 @@
         <v>46219</v>
       </c>
       <c r="M16" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
@@ -1592,7 +1592,7 @@
         <v>46219</v>
       </c>
       <c r="M17" s="4" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
chore: back up company tracking 2026-09-01
</commit_message>
<xml_diff>
--- a/watchlists/a_share_company_watchlist.xlsx
+++ b/watchlists/a_share_company_watchlist.xlsx
@@ -594,7 +594,7 @@
         <v>46151</v>
       </c>
       <c r="M2" s="4" t="n">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
@@ -796,7 +796,7 @@
         <v>46151</v>
       </c>
       <c r="M5" s="4" t="n">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
@@ -862,7 +862,7 @@
         <v>46151</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
@@ -928,7 +928,7 @@
         <v>46151</v>
       </c>
       <c r="M7" s="4" t="n">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
@@ -994,7 +994,7 @@
         <v>46151</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
@@ -1060,7 +1060,7 @@
         <v>46151</v>
       </c>
       <c r="M9" s="4" t="n">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
@@ -1126,7 +1126,7 @@
         <v>46151</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
@@ -1192,7 +1192,7 @@
         <v>46156</v>
       </c>
       <c r="M11" s="4" t="n">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
@@ -1258,7 +1258,7 @@
         <v>46156</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
@@ -1394,7 +1394,7 @@
         <v>46181</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
@@ -1460,7 +1460,7 @@
         <v>46205</v>
       </c>
       <c r="M15" s="4" t="n">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
@@ -1526,7 +1526,7 @@
         <v>46219</v>
       </c>
       <c r="M16" s="4" t="n">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
@@ -1592,7 +1592,7 @@
         <v>46219</v>
       </c>
       <c r="M17" s="4" t="n">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
chore: back up company tracking 2026-09-02
</commit_message>
<xml_diff>
--- a/watchlists/a_share_company_watchlist.xlsx
+++ b/watchlists/a_share_company_watchlist.xlsx
@@ -594,7 +594,7 @@
         <v>46151</v>
       </c>
       <c r="M2" s="4" t="n">
-        <v>46266</v>
+        <v>46267</v>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
@@ -796,7 +796,7 @@
         <v>46151</v>
       </c>
       <c r="M5" s="4" t="n">
-        <v>46266</v>
+        <v>46267</v>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
@@ -862,7 +862,7 @@
         <v>46151</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>46266</v>
+        <v>46267</v>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
@@ -928,7 +928,7 @@
         <v>46151</v>
       </c>
       <c r="M7" s="4" t="n">
-        <v>46266</v>
+        <v>46267</v>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
@@ -994,7 +994,7 @@
         <v>46151</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>46266</v>
+        <v>46267</v>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
@@ -1060,7 +1060,7 @@
         <v>46151</v>
       </c>
       <c r="M9" s="4" t="n">
-        <v>46266</v>
+        <v>46267</v>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
@@ -1126,7 +1126,7 @@
         <v>46151</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>46266</v>
+        <v>46267</v>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
@@ -1192,7 +1192,7 @@
         <v>46156</v>
       </c>
       <c r="M11" s="4" t="n">
-        <v>46266</v>
+        <v>46267</v>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
@@ -1258,7 +1258,7 @@
         <v>46156</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>46266</v>
+        <v>46267</v>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
@@ -1394,7 +1394,7 @@
         <v>46181</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>46266</v>
+        <v>46267</v>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
@@ -1460,7 +1460,7 @@
         <v>46205</v>
       </c>
       <c r="M15" s="4" t="n">
-        <v>46266</v>
+        <v>46267</v>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
@@ -1526,7 +1526,7 @@
         <v>46219</v>
       </c>
       <c r="M16" s="4" t="n">
-        <v>46266</v>
+        <v>46267</v>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
@@ -1592,7 +1592,7 @@
         <v>46219</v>
       </c>
       <c r="M17" s="4" t="n">
-        <v>46266</v>
+        <v>46267</v>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
chore: back up company tracking 2026-09-03
</commit_message>
<xml_diff>
--- a/watchlists/a_share_company_watchlist.xlsx
+++ b/watchlists/a_share_company_watchlist.xlsx
@@ -594,7 +594,7 @@
         <v>46151</v>
       </c>
       <c r="M2" s="4" t="n">
-        <v>46267</v>
+        <v>46268</v>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
@@ -796,7 +796,7 @@
         <v>46151</v>
       </c>
       <c r="M5" s="4" t="n">
-        <v>46267</v>
+        <v>46268</v>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
@@ -862,7 +862,7 @@
         <v>46151</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>46267</v>
+        <v>46268</v>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
@@ -928,7 +928,7 @@
         <v>46151</v>
       </c>
       <c r="M7" s="4" t="n">
-        <v>46267</v>
+        <v>46268</v>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
@@ -994,7 +994,7 @@
         <v>46151</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>46267</v>
+        <v>46268</v>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
@@ -1060,7 +1060,7 @@
         <v>46151</v>
       </c>
       <c r="M9" s="4" t="n">
-        <v>46267</v>
+        <v>46268</v>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
@@ -1126,7 +1126,7 @@
         <v>46151</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>46267</v>
+        <v>46268</v>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
@@ -1192,7 +1192,7 @@
         <v>46156</v>
       </c>
       <c r="M11" s="4" t="n">
-        <v>46267</v>
+        <v>46268</v>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
@@ -1258,7 +1258,7 @@
         <v>46156</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>46267</v>
+        <v>46268</v>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
@@ -1394,7 +1394,7 @@
         <v>46181</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>46267</v>
+        <v>46268</v>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
@@ -1460,7 +1460,7 @@
         <v>46205</v>
       </c>
       <c r="M15" s="4" t="n">
-        <v>46267</v>
+        <v>46268</v>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
@@ -1526,7 +1526,7 @@
         <v>46219</v>
       </c>
       <c r="M16" s="4" t="n">
-        <v>46267</v>
+        <v>46268</v>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
@@ -1592,7 +1592,7 @@
         <v>46219</v>
       </c>
       <c r="M17" s="4" t="n">
-        <v>46267</v>
+        <v>46268</v>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
chore: back up company tracking 2026-09-05
</commit_message>
<xml_diff>
--- a/watchlists/a_share_company_watchlist.xlsx
+++ b/watchlists/a_share_company_watchlist.xlsx
@@ -594,7 +594,7 @@
         <v>46151</v>
       </c>
       <c r="M2" s="4" t="n">
-        <v>46268</v>
+        <v>46270</v>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
@@ -796,7 +796,7 @@
         <v>46151</v>
       </c>
       <c r="M5" s="4" t="n">
-        <v>46268</v>
+        <v>46270</v>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
@@ -862,7 +862,7 @@
         <v>46151</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>46268</v>
+        <v>46270</v>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
@@ -928,7 +928,7 @@
         <v>46151</v>
       </c>
       <c r="M7" s="4" t="n">
-        <v>46268</v>
+        <v>46270</v>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
@@ -994,7 +994,7 @@
         <v>46151</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>46268</v>
+        <v>46270</v>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
@@ -1060,7 +1060,7 @@
         <v>46151</v>
       </c>
       <c r="M9" s="4" t="n">
-        <v>46268</v>
+        <v>46270</v>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
@@ -1126,7 +1126,7 @@
         <v>46151</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>46268</v>
+        <v>46270</v>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
@@ -1192,7 +1192,7 @@
         <v>46156</v>
       </c>
       <c r="M11" s="4" t="n">
-        <v>46268</v>
+        <v>46270</v>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
@@ -1258,7 +1258,7 @@
         <v>46156</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>46268</v>
+        <v>46270</v>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
@@ -1394,7 +1394,7 @@
         <v>46181</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>46268</v>
+        <v>46270</v>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
@@ -1460,7 +1460,7 @@
         <v>46205</v>
       </c>
       <c r="M15" s="4" t="n">
-        <v>46268</v>
+        <v>46270</v>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
@@ -1526,7 +1526,7 @@
         <v>46219</v>
       </c>
       <c r="M16" s="4" t="n">
-        <v>46268</v>
+        <v>46270</v>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
@@ -1592,7 +1592,7 @@
         <v>46219</v>
       </c>
       <c r="M17" s="4" t="n">
-        <v>46268</v>
+        <v>46270</v>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>

</xml_diff>